<commit_message>
add step by step evidence PDF
</commit_message>
<xml_diff>
--- a/student_performance_knime.xlsx
+++ b/student_performance_knime.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/870a9848b561422d/Desktop/DemoEarlyWarningTool/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0821F8DB-7B8F-4D65-B038-BC10FF2ACB49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="8_{0821F8DB-7B8F-4D65-B038-BC10FF2ACB49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{71DA5DA9-DE21-4486-A9CF-5841D451456B}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{31502626-4C06-41BB-ACA5-07A9E0BC727E}"/>
+    <workbookView xWindow="3855" yWindow="3855" windowWidth="21600" windowHeight="11775" xr2:uid="{31502626-4C06-41BB-ACA5-07A9E0BC727E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,15 +38,140 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="38">
+  <si>
+    <t>student_id</t>
+  </si>
+  <si>
+    <t>attendance</t>
+  </si>
+  <si>
+    <t>quiz_score</t>
+  </si>
+  <si>
+    <t>assignment_score</t>
+  </si>
+  <si>
+    <t>exam_score</t>
+  </si>
+  <si>
+    <t>risk_status</t>
+  </si>
+  <si>
+    <t>S001</t>
+  </si>
+  <si>
+    <t>Not At Risk</t>
+  </si>
+  <si>
+    <t>S002</t>
+  </si>
+  <si>
+    <t>S003</t>
+  </si>
+  <si>
+    <t>S004</t>
+  </si>
+  <si>
+    <t>At Risk</t>
+  </si>
+  <si>
+    <t>S005</t>
+  </si>
+  <si>
+    <t>S006</t>
+  </si>
+  <si>
+    <t>S007</t>
+  </si>
+  <si>
+    <t>S008</t>
+  </si>
+  <si>
+    <t>S009</t>
+  </si>
+  <si>
+    <t>S010</t>
+  </si>
+  <si>
+    <t>S011</t>
+  </si>
+  <si>
+    <t>S012</t>
+  </si>
+  <si>
+    <t>S013</t>
+  </si>
+  <si>
+    <t>S014</t>
+  </si>
+  <si>
+    <t>S015</t>
+  </si>
+  <si>
+    <t>S016</t>
+  </si>
+  <si>
+    <t>S017</t>
+  </si>
+  <si>
+    <t>S018</t>
+  </si>
+  <si>
+    <t>S019</t>
+  </si>
+  <si>
+    <t>S020</t>
+  </si>
+  <si>
+    <t>S021</t>
+  </si>
+  <si>
+    <t>S022</t>
+  </si>
+  <si>
+    <t>S023</t>
+  </si>
+  <si>
+    <t>S024</t>
+  </si>
+  <si>
+    <t>S025</t>
+  </si>
+  <si>
+    <t>S026</t>
+  </si>
+  <si>
+    <t>S027</t>
+  </si>
+  <si>
+    <t>S028</t>
+  </si>
+  <si>
+    <t>S029</t>
+  </si>
+  <si>
+    <t>S030</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -69,8 +194,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -405,9 +531,630 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D55CED3-40D7-48EB-B38D-ED3ADCECFB7F}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="1">
+        <v>95</v>
+      </c>
+      <c r="C2" s="1">
+        <v>90</v>
+      </c>
+      <c r="D2" s="1">
+        <v>92</v>
+      </c>
+      <c r="E2" s="1">
+        <v>88</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="1">
+        <v>88</v>
+      </c>
+      <c r="C3" s="1">
+        <v>84</v>
+      </c>
+      <c r="D3" s="1">
+        <v>86</v>
+      </c>
+      <c r="E3" s="1">
+        <v>82</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="1">
+        <v>76</v>
+      </c>
+      <c r="C4" s="1">
+        <v>72</v>
+      </c>
+      <c r="D4" s="1">
+        <v>75</v>
+      </c>
+      <c r="E4" s="1">
+        <v>70</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="1">
+        <v>62</v>
+      </c>
+      <c r="C5" s="1">
+        <v>58</v>
+      </c>
+      <c r="D5" s="1">
+        <v>60</v>
+      </c>
+      <c r="E5" s="1">
+        <v>55</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="1">
+        <v>55</v>
+      </c>
+      <c r="C6" s="1">
+        <v>48</v>
+      </c>
+      <c r="D6" s="1">
+        <v>52</v>
+      </c>
+      <c r="E6" s="1">
+        <v>50</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="1">
+        <v>91</v>
+      </c>
+      <c r="C7" s="1">
+        <v>87</v>
+      </c>
+      <c r="D7" s="1">
+        <v>89</v>
+      </c>
+      <c r="E7" s="1">
+        <v>85</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="1">
+        <v>68</v>
+      </c>
+      <c r="C8" s="1">
+        <v>65</v>
+      </c>
+      <c r="D8" s="1">
+        <v>61</v>
+      </c>
+      <c r="E8" s="1">
+        <v>60</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="1">
+        <v>82</v>
+      </c>
+      <c r="C9" s="1">
+        <v>78</v>
+      </c>
+      <c r="D9" s="1">
+        <v>80</v>
+      </c>
+      <c r="E9" s="1">
+        <v>76</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="1">
+        <v>47</v>
+      </c>
+      <c r="C10" s="1">
+        <v>50</v>
+      </c>
+      <c r="D10" s="1">
+        <v>45</v>
+      </c>
+      <c r="E10" s="1">
+        <v>48</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="1">
+        <v>73</v>
+      </c>
+      <c r="C11" s="1">
+        <v>69</v>
+      </c>
+      <c r="D11" s="1">
+        <v>72</v>
+      </c>
+      <c r="E11" s="1">
+        <v>68</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="1">
+        <v>85</v>
+      </c>
+      <c r="C12" s="1">
+        <v>81</v>
+      </c>
+      <c r="D12" s="1">
+        <v>79</v>
+      </c>
+      <c r="E12" s="1">
+        <v>83</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" s="1">
+        <v>59</v>
+      </c>
+      <c r="C13" s="1">
+        <v>55</v>
+      </c>
+      <c r="D13" s="1">
+        <v>57</v>
+      </c>
+      <c r="E13" s="1">
+        <v>52</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="1">
+        <v>79</v>
+      </c>
+      <c r="C14" s="1">
+        <v>74</v>
+      </c>
+      <c r="D14" s="1">
+        <v>77</v>
+      </c>
+      <c r="E14" s="1">
+        <v>73</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" s="1">
+        <v>66</v>
+      </c>
+      <c r="C15" s="1">
+        <v>62</v>
+      </c>
+      <c r="D15" s="1">
+        <v>64</v>
+      </c>
+      <c r="E15" s="1">
+        <v>58</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16" s="1">
+        <v>93</v>
+      </c>
+      <c r="C16" s="1">
+        <v>92</v>
+      </c>
+      <c r="D16" s="1">
+        <v>90</v>
+      </c>
+      <c r="E16" s="1">
+        <v>91</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B17" s="1">
+        <v>71</v>
+      </c>
+      <c r="C17" s="1">
+        <v>67</v>
+      </c>
+      <c r="D17" s="1">
+        <v>69</v>
+      </c>
+      <c r="E17" s="1">
+        <v>65</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B18" s="1">
+        <v>87</v>
+      </c>
+      <c r="C18" s="1">
+        <v>83</v>
+      </c>
+      <c r="D18" s="1">
+        <v>85</v>
+      </c>
+      <c r="E18" s="1">
+        <v>80</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B19" s="1">
+        <v>52</v>
+      </c>
+      <c r="C19" s="1">
+        <v>46</v>
+      </c>
+      <c r="D19" s="1">
+        <v>49</v>
+      </c>
+      <c r="E19" s="1">
+        <v>44</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" s="1">
+        <v>74</v>
+      </c>
+      <c r="C20" s="1">
+        <v>71</v>
+      </c>
+      <c r="D20" s="1">
+        <v>73</v>
+      </c>
+      <c r="E20" s="1">
+        <v>69</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B21" s="1">
+        <v>64</v>
+      </c>
+      <c r="C21" s="1">
+        <v>59</v>
+      </c>
+      <c r="D21" s="1">
+        <v>62</v>
+      </c>
+      <c r="E21" s="1">
+        <v>56</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B22" s="1">
+        <v>89</v>
+      </c>
+      <c r="C22" s="1">
+        <v>86</v>
+      </c>
+      <c r="D22" s="1">
+        <v>88</v>
+      </c>
+      <c r="E22" s="1">
+        <v>84</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B23" s="1">
+        <v>57</v>
+      </c>
+      <c r="C23" s="1">
+        <v>53</v>
+      </c>
+      <c r="D23" s="1">
+        <v>55</v>
+      </c>
+      <c r="E23" s="1">
+        <v>49</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B24" s="1">
+        <v>81</v>
+      </c>
+      <c r="C24" s="1">
+        <v>76</v>
+      </c>
+      <c r="D24" s="1">
+        <v>78</v>
+      </c>
+      <c r="E24" s="1">
+        <v>75</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B25" s="1">
+        <v>69</v>
+      </c>
+      <c r="C25" s="1">
+        <v>64</v>
+      </c>
+      <c r="D25" s="1">
+        <v>66</v>
+      </c>
+      <c r="E25" s="1">
+        <v>61</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B26" s="1">
+        <v>96</v>
+      </c>
+      <c r="C26" s="1">
+        <v>94</v>
+      </c>
+      <c r="D26" s="1">
+        <v>93</v>
+      </c>
+      <c r="E26" s="1">
+        <v>95</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B27" s="1">
+        <v>61</v>
+      </c>
+      <c r="C27" s="1">
+        <v>57</v>
+      </c>
+      <c r="D27" s="1">
+        <v>59</v>
+      </c>
+      <c r="E27" s="1">
+        <v>54</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B28" s="1">
+        <v>78</v>
+      </c>
+      <c r="C28" s="1">
+        <v>73</v>
+      </c>
+      <c r="D28" s="1">
+        <v>76</v>
+      </c>
+      <c r="E28" s="1">
+        <v>72</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B29" s="1">
+        <v>49</v>
+      </c>
+      <c r="C29" s="1">
+        <v>44</v>
+      </c>
+      <c r="D29" s="1">
+        <v>47</v>
+      </c>
+      <c r="E29" s="1">
+        <v>42</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B30" s="1">
+        <v>84</v>
+      </c>
+      <c r="C30" s="1">
+        <v>80</v>
+      </c>
+      <c r="D30" s="1">
+        <v>82</v>
+      </c>
+      <c r="E30" s="1">
+        <v>79</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B31" s="1">
+        <v>72</v>
+      </c>
+      <c r="C31" s="1">
+        <v>66</v>
+      </c>
+      <c r="D31" s="1">
+        <v>68</v>
+      </c>
+      <c r="E31" s="1">
+        <v>63</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>